<commit_message>
UI board piece rendering
</commit_message>
<xml_diff>
--- a/Sprint 1 Task Assignments.xlsx
+++ b/Sprint 1 Task Assignments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/219b9449e9f9313b/Desktop/CPTS 322/Chess-Bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{4C77C863-50A8-44CE-B033-22D8A9EBDD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7747AE88-3D43-4547-A21F-0E07253510B4}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{4C77C863-50A8-44CE-B033-22D8A9EBDD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EE62579-EE05-43A4-9341-601679AF2954}"/>
   <bookViews>
     <workbookView xWindow="23052" yWindow="12" windowWidth="23016" windowHeight="13656" xr2:uid="{53B90E79-2679-4896-BE69-64556766AB64}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="33">
   <si>
     <t>Task</t>
   </si>
@@ -702,19 +702,21 @@
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="3"/>
+      <c r="C10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">

</xml_diff>

<commit_message>
UI command handler and GameController start
</commit_message>
<xml_diff>
--- a/Sprint 1 Task Assignments.xlsx
+++ b/Sprint 1 Task Assignments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/219b9449e9f9313b/Desktop/CPTS 322/Chess-Bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{4C77C863-50A8-44CE-B033-22D8A9EBDD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EE62579-EE05-43A4-9341-601679AF2954}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{4C77C863-50A8-44CE-B033-22D8A9EBDD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4144C8B2-D016-4537-87FC-97A2DD904466}"/>
   <bookViews>
     <workbookView xWindow="23052" yWindow="12" windowWidth="23016" windowHeight="13656" xr2:uid="{53B90E79-2679-4896-BE69-64556766AB64}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
   <si>
     <t>Task</t>
   </si>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <t>Added Chess pieces and populate boards init state</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Pipeline, not game logic</t>
   </si>
 </sst>
 </file>
@@ -541,6 +547,7 @@
     <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -560,6 +567,9 @@
       <c r="E1" t="s">
         <v>22</v>
       </c>
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -694,12 +704,17 @@
         <v>10</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -777,16 +792,19 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="C16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finished sprint 1 documentation
</commit_message>
<xml_diff>
--- a/Sprint 1 Task Assignments.xlsx
+++ b/Sprint 1 Task Assignments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/219b9449e9f9313b/Desktop/CPTS 322/Chess-Bot/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files Code\CPTS 322 Code\Chess-Bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{4C77C863-50A8-44CE-B033-22D8A9EBDD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4144C8B2-D016-4537-87FC-97A2DD904466}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E54E3F9E-92DD-48D5-93A3-3776217B87A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23052" yWindow="12" windowWidth="23016" windowHeight="13656" xr2:uid="{53B90E79-2679-4896-BE69-64556766AB64}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53B90E79-2679-4896-BE69-64556766AB64}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="37">
   <si>
     <t>Task</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>Pipeline, not game logic</t>
+  </si>
+  <si>
+    <t>Issac</t>
+  </si>
+  <si>
+    <t>Isaac &amp; Johnny</t>
   </si>
 </sst>
 </file>
@@ -541,17 +547,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F8B371-8FC1-4A7E-9445-FCA167F673D1}">
   <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -571,7 +577,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -600,7 +606,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -608,10 +614,13 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -628,7 +637,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -645,7 +654,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -662,7 +671,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -679,7 +688,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -696,7 +705,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -716,7 +725,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -733,49 +742,58 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C11" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="E11" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="E12" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="C13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E13" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -783,7 +801,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -791,7 +809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
@@ -808,7 +826,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -822,7 +840,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>20</v>
       </c>

</xml_diff>